<commit_message>
Add robust regressors; explain missing optional boosters
- Expand model suite with robust + Bayesian + kernel ridge regressors (sklearn-only)
- Log why LightGBM/XGBoost/CatBoost folders may be absent (optional boosters disabled by default)
- Regenerate outputs for new models

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/outputs/models/tables/all_model_metrics.xlsx
+++ b/outputs/models/tables/all_model_metrics.xlsx
@@ -13,27 +13,33 @@
     <sheet name="metrics__Ridge Regression" sheetId="4" r:id="rId4"/>
     <sheet name="metrics__Lasso Regression" sheetId="5" r:id="rId5"/>
     <sheet name="metrics__Elastic Net Regression" sheetId="6" r:id="rId6"/>
-    <sheet name="metrics__Polynomial Regression " sheetId="7" r:id="rId7"/>
-    <sheet name="metrics__Polynomial Ridge Degre" sheetId="8" r:id="rId8"/>
-    <sheet name="metrics__Stochastic Gradient Re" sheetId="9" r:id="rId9"/>
-    <sheet name="metrics__Decision Tree" sheetId="10" r:id="rId10"/>
-    <sheet name="metrics__Random Forest" sheetId="11" r:id="rId11"/>
-    <sheet name="metrics__Extra Trees" sheetId="12" r:id="rId12"/>
-    <sheet name="metrics__Gradient Boosting" sheetId="13" r:id="rId13"/>
-    <sheet name="metrics__Adaptive Boosting" sheetId="14" r:id="rId14"/>
-    <sheet name="metrics__Histogram Gradient Boo" sheetId="15" r:id="rId15"/>
-    <sheet name="metrics__Bagging Regressor" sheetId="16" r:id="rId16"/>
-    <sheet name="metrics__K Nearest Neighbors Fi" sheetId="17" r:id="rId17"/>
-    <sheet name="metrics__K Nearest Neighbors Th" sheetId="18" r:id="rId18"/>
-    <sheet name="metrics__Support Vector Regress" sheetId="19" r:id="rId19"/>
-    <sheet name="metrics__Gaussian Process Regre" sheetId="20" r:id="rId20"/>
+    <sheet name="metrics__Huber Regression" sheetId="7" r:id="rId7"/>
+    <sheet name="metrics__Theil Sen Regression" sheetId="8" r:id="rId8"/>
+    <sheet name="metrics__RANSAC Regression" sheetId="9" r:id="rId9"/>
+    <sheet name="metrics__Bayesian Ridge Regress" sheetId="10" r:id="rId10"/>
+    <sheet name="metrics__ARD Regression" sheetId="11" r:id="rId11"/>
+    <sheet name="metrics__Polynomial Regression " sheetId="12" r:id="rId12"/>
+    <sheet name="metrics__Polynomial Ridge Degre" sheetId="13" r:id="rId13"/>
+    <sheet name="metrics__Stochastic Gradient Re" sheetId="14" r:id="rId14"/>
+    <sheet name="metrics__Kernel Ridge Regressio" sheetId="15" r:id="rId15"/>
+    <sheet name="metrics__Decision Tree" sheetId="16" r:id="rId16"/>
+    <sheet name="metrics__Random Forest" sheetId="17" r:id="rId17"/>
+    <sheet name="metrics__Extra Trees" sheetId="18" r:id="rId18"/>
+    <sheet name="metrics__Gradient Boosting" sheetId="19" r:id="rId19"/>
+    <sheet name="metrics__Adaptive Boosting" sheetId="20" r:id="rId20"/>
+    <sheet name="metrics__Histogram Gradient Boo" sheetId="21" r:id="rId21"/>
+    <sheet name="metrics__Bagging Regressor" sheetId="22" r:id="rId22"/>
+    <sheet name="metrics__K Nearest Neighbors Fi" sheetId="23" r:id="rId23"/>
+    <sheet name="metrics__K Nearest Neighbors Th" sheetId="24" r:id="rId24"/>
+    <sheet name="metrics__Support Vector Regress" sheetId="25" r:id="rId25"/>
+    <sheet name="metrics__Gaussian Process Regre" sheetId="26" r:id="rId26"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="48">
   <si>
     <t>model</t>
   </si>
@@ -101,6 +107,15 @@
     <t>Ridge Regression</t>
   </si>
   <si>
+    <t>Bayesian Ridge Regression</t>
+  </si>
+  <si>
+    <t>ARD Regression</t>
+  </si>
+  <si>
+    <t>Huber Regression</t>
+  </si>
+  <si>
     <t>K Nearest Neighbors Five</t>
   </si>
   <si>
@@ -111,6 +126,15 @@
   </si>
   <si>
     <t>Histogram Gradient Boosting</t>
+  </si>
+  <si>
+    <t>Kernel Ridge Regression</t>
+  </si>
+  <si>
+    <t>Theil Sen Regression</t>
+  </si>
+  <si>
+    <t>RANSAC Regression</t>
   </si>
   <si>
     <t>Stochastic Gradient Regression</t>
@@ -516,7 +540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -892,19 +916,19 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>20.55809523809524</v>
+        <v>17.56917343216907</v>
       </c>
       <c r="C17">
-        <v>29.28115086549835</v>
+        <v>24.13531616499252</v>
       </c>
       <c r="D17">
-        <v>0.09571559727788351</v>
+        <v>0.3236340906910181</v>
       </c>
       <c r="E17">
-        <v>0.02035856371770714</v>
+        <v>0.2672702649152696</v>
       </c>
       <c r="F17">
-        <v>38.56851652347636</v>
+        <v>38.33727603024025</v>
       </c>
       <c r="G17">
         <v>16</v>
@@ -915,19 +939,19 @@
         <v>23</v>
       </c>
       <c r="B18">
-        <v>20.55809523809524</v>
+        <v>17.56917343216907</v>
       </c>
       <c r="C18">
-        <v>29.28115086549835</v>
+        <v>24.13531616499252</v>
       </c>
       <c r="D18">
-        <v>0.09571559727788351</v>
+        <v>0.3236340906910181</v>
       </c>
       <c r="E18">
-        <v>0.02035856371770714</v>
+        <v>0.2672702649152696</v>
       </c>
       <c r="F18">
-        <v>38.56851652347636</v>
+        <v>38.33727603024025</v>
       </c>
       <c r="G18">
         <v>17</v>
@@ -938,19 +962,19 @@
         <v>24</v>
       </c>
       <c r="B19">
-        <v>21.08132541145396</v>
+        <v>16.2715137120993</v>
       </c>
       <c r="C19">
-        <v>29.78566177295085</v>
+        <v>24.81725687316666</v>
       </c>
       <c r="D19">
-        <v>0.06338891693132301</v>
+        <v>0.2815534835374435</v>
       </c>
       <c r="E19">
-        <v>-0.2175944079892801</v>
+        <v>0.2216829404988971</v>
       </c>
       <c r="F19">
-        <v>49.73564455388451</v>
+        <v>37.85555828845195</v>
       </c>
       <c r="G19">
         <v>18</v>
@@ -961,19 +985,19 @@
         <v>25</v>
       </c>
       <c r="B20">
-        <v>21.80005102040816</v>
+        <v>20.55809523809524</v>
       </c>
       <c r="C20">
-        <v>30.8200775199298</v>
+        <v>29.28115086549835</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>0.09571559727788351</v>
       </c>
       <c r="E20">
-        <v>-0.08333333333333326</v>
+        <v>0.02035856371770714</v>
       </c>
       <c r="F20">
-        <v>51.86540618403083</v>
+        <v>38.56851652347636</v>
       </c>
       <c r="G20">
         <v>19</v>
@@ -984,22 +1008,160 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>56.87433699333061</v>
+        <v>20.55809523809524</v>
       </c>
       <c r="C21">
-        <v>62.66107261418601</v>
+        <v>29.28115086549835</v>
       </c>
       <c r="D21">
-        <v>-3.36311947070695</v>
+        <v>0.09571559727788351</v>
       </c>
       <c r="E21">
-        <v>-3.726712759932529</v>
+        <v>0.02035856371770714</v>
       </c>
       <c r="F21">
-        <v>48.04105268799751</v>
+        <v>38.56851652347636</v>
       </c>
       <c r="G21">
         <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22">
+        <v>21.08132541145396</v>
+      </c>
+      <c r="C22">
+        <v>29.78566177295085</v>
+      </c>
+      <c r="D22">
+        <v>0.06338891693132301</v>
+      </c>
+      <c r="E22">
+        <v>-0.2175944079892801</v>
+      </c>
+      <c r="F22">
+        <v>49.73564455388451</v>
+      </c>
+      <c r="G22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23">
+        <v>21.80005102040816</v>
+      </c>
+      <c r="C23">
+        <v>30.8200775199298</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>-0.08333333333333326</v>
+      </c>
+      <c r="F23">
+        <v>51.86540618403083</v>
+      </c>
+      <c r="G23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24">
+        <v>26.70499493863093</v>
+      </c>
+      <c r="C24">
+        <v>31.86005853528316</v>
+      </c>
+      <c r="D24">
+        <v>-0.1756461895250861</v>
+      </c>
+      <c r="E24">
+        <v>-0.2736167053188433</v>
+      </c>
+      <c r="F24">
+        <v>35.60357253216966</v>
+      </c>
+      <c r="G24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25">
+        <v>20.29500914141204</v>
+      </c>
+      <c r="C25">
+        <v>33.81975526068013</v>
+      </c>
+      <c r="D25">
+        <v>-0.1806837958833397</v>
+      </c>
+      <c r="E25">
+        <v>-0.2790741122069513</v>
+      </c>
+      <c r="F25">
+        <v>38.36346684702566</v>
+      </c>
+      <c r="G25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26">
+        <v>20.1202592296975</v>
+      </c>
+      <c r="C26">
+        <v>34.99768010898507</v>
+      </c>
+      <c r="D26">
+        <v>-1.027851374414385</v>
+      </c>
+      <c r="E26">
+        <v>-1.196838988948917</v>
+      </c>
+      <c r="F26">
+        <v>56.06014171810725</v>
+      </c>
+      <c r="G26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27">
+        <v>56.87433699333061</v>
+      </c>
+      <c r="C27">
+        <v>62.66107261418601</v>
+      </c>
+      <c r="D27">
+        <v>-3.36311947070695</v>
+      </c>
+      <c r="E27">
+        <v>-3.726712759932529</v>
+      </c>
+      <c r="F27">
+        <v>48.04105268799751</v>
+      </c>
+      <c r="G27">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1014,176 +1176,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>11.18523809523809</v>
+        <v>18.09743140653623</v>
       </c>
       <c r="C2">
-        <v>201.3859261904761</v>
+        <v>470.6185449835385</v>
       </c>
       <c r="D2">
-        <v>14.19105091917002</v>
+        <v>21.6937443744398</v>
       </c>
       <c r="E2">
-        <v>0.8803477478228072</v>
+        <v>0.7203847861226714</v>
       </c>
       <c r="F2">
-        <v>0.8703767268080411</v>
+        <v>0.6970835182995607</v>
       </c>
       <c r="G2">
-        <v>58.07192754245103</v>
+        <v>102.4514769731611</v>
       </c>
       <c r="H2">
-        <v>9.435833333333328</v>
+        <v>15.75634632822069</v>
       </c>
       <c r="I2">
-        <v>0.8803477478228072</v>
+        <v>0.7203847861226714</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>4.207142857142858</v>
+        <v>9.353700830464478</v>
       </c>
       <c r="C3">
-        <v>23.39107142857144</v>
+        <v>159.3046109319126</v>
       </c>
       <c r="D3">
-        <v>4.83643168343888</v>
+        <v>12.62159304255658</v>
       </c>
       <c r="E3">
-        <v>0.8531707765440903</v>
+        <v>2.133773540125006E-05</v>
       </c>
       <c r="F3">
-        <v>0.8409350079227645</v>
+        <v>-0.08331021745331535</v>
       </c>
       <c r="G3">
-        <v>7.268140300799806</v>
+        <v>17.74260092367239</v>
       </c>
       <c r="H3">
-        <v>3.524999999999999</v>
+        <v>7.064082669368744</v>
       </c>
       <c r="I3">
-        <v>0.8531707765440903</v>
+        <v>2.13377354014721E-05</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>15.00714285714286</v>
+        <v>32.1031453166423</v>
       </c>
       <c r="C4">
-        <v>336.815773809524</v>
+        <v>2334.071474360047</v>
       </c>
       <c r="D4">
-        <v>18.35254134471638</v>
+        <v>48.31222903530789</v>
       </c>
       <c r="E4">
-        <v>0.8556964367356024</v>
+        <v>2.800182344775415E-06</v>
       </c>
       <c r="F4">
-        <v>0.8436711397969026</v>
+        <v>-0.08333029980245987</v>
       </c>
       <c r="G4">
-        <v>6.80814351818554</v>
+        <v>16.64107669905803</v>
       </c>
       <c r="H4">
-        <v>15.44583333333333</v>
+        <v>22.53605311998928</v>
       </c>
       <c r="I4">
-        <v>0.8556964367356024</v>
+        <v>2.800182344664393E-06</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>7.223809523809522</v>
+        <v>10.72241617503328</v>
       </c>
       <c r="C5">
-        <v>105.027619047619</v>
+        <v>193.5909978140026</v>
       </c>
       <c r="D5">
-        <v>10.24829834887817</v>
+        <v>13.9136982076658</v>
       </c>
       <c r="E5">
-        <v>0.7689542301365704</v>
+        <v>0.574127438723655</v>
       </c>
       <c r="F5">
-        <v>0.7497004159812846</v>
+        <v>0.538638058617293</v>
       </c>
       <c r="G5">
-        <v>11.21539909324933</v>
+        <v>16.5139495250695</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>0.7689542301365704</v>
+        <v>0.574127438723655</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>9.405833333333334</v>
+        <v>17.56917343216907</v>
       </c>
       <c r="C6">
-        <v>166.6550976190477</v>
+        <v>789.3964070223751</v>
       </c>
       <c r="D6">
-        <v>11.90708057405086</v>
+        <v>24.13531616499252</v>
       </c>
       <c r="E6">
-        <v>0.8395422978097675</v>
+        <v>0.3236340906910181</v>
       </c>
       <c r="F6">
-        <v>0.8261708226272482</v>
+        <v>0.2672702649152696</v>
       </c>
       <c r="G6">
-        <v>20.84090261367143</v>
+        <v>38.33727603024025</v>
       </c>
       <c r="H6">
-        <v>8.351666666666663</v>
+        <v>13.83912052939468</v>
       </c>
       <c r="I6">
-        <v>0.8395422978097675</v>
+        <v>0.3236340906910181</v>
       </c>
     </row>
   </sheetData>
@@ -1198,176 +1360,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>11.20179695011338</v>
+        <v>18.09743140653623</v>
       </c>
       <c r="C2">
-        <v>224.7096343972572</v>
+        <v>470.6185449835385</v>
       </c>
       <c r="D2">
-        <v>14.99031802188523</v>
+        <v>21.6937443744398</v>
       </c>
       <c r="E2">
-        <v>0.8664901050924733</v>
+        <v>0.7203847861226714</v>
       </c>
       <c r="F2">
-        <v>0.855364280516846</v>
+        <v>0.6970835182995607</v>
       </c>
       <c r="G2">
-        <v>58.90464254253096</v>
+        <v>102.451476973161</v>
       </c>
       <c r="H2">
-        <v>8.386608544973544</v>
+        <v>15.75634632822069</v>
       </c>
       <c r="I2">
-        <v>0.8678324828815218</v>
+        <v>0.7203847861226714</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>4.73816678004534</v>
+        <v>9.353700830464478</v>
       </c>
       <c r="C3">
-        <v>42.66476898952453</v>
+        <v>159.3046109319126</v>
       </c>
       <c r="D3">
-        <v>6.531827385159878</v>
+        <v>12.62159304255658</v>
       </c>
       <c r="E3">
-        <v>0.7321869193214529</v>
+        <v>2.133773540125006E-05</v>
       </c>
       <c r="F3">
-        <v>0.7098691625982405</v>
+        <v>-0.08331021745331535</v>
       </c>
       <c r="G3">
-        <v>8.831622888899272</v>
+        <v>17.74260092367239</v>
       </c>
       <c r="H3">
-        <v>3.799534920634933</v>
+        <v>7.064082669368744</v>
       </c>
       <c r="I3">
-        <v>0.7323021588655974</v>
+        <v>2.13377354014721E-05</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>19.56376118154327</v>
+        <v>32.1031453166423</v>
       </c>
       <c r="C4">
-        <v>621.5268394215173</v>
+        <v>2334.071474360047</v>
       </c>
       <c r="D4">
-        <v>24.93044001660455</v>
+        <v>48.31222903530789</v>
       </c>
       <c r="E4">
-        <v>0.7337163382267701</v>
+        <v>2.800182344775415E-06</v>
       </c>
       <c r="F4">
-        <v>0.711526033079001</v>
+        <v>-0.08333029980245987</v>
       </c>
       <c r="G4">
-        <v>9.410596220698149</v>
+        <v>16.64107669905803</v>
       </c>
       <c r="H4">
-        <v>17.369032539682</v>
+        <v>22.53605311998928</v>
       </c>
       <c r="I4">
-        <v>0.7337254489870485</v>
+        <v>2.800182344664393E-06</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>7.093999470899462</v>
+        <v>10.72241617503328</v>
       </c>
       <c r="C5">
-        <v>107.2273667275214</v>
+        <v>193.5909978140027</v>
       </c>
       <c r="D5">
-        <v>10.35506478625418</v>
+        <v>13.91369820766581</v>
       </c>
       <c r="E5">
-        <v>0.7641150992411256</v>
+        <v>0.5741274387236548</v>
       </c>
       <c r="F5">
-        <v>0.7444580241778862</v>
+        <v>0.5386380586172927</v>
       </c>
       <c r="G5">
-        <v>11.83427841832139</v>
+        <v>16.51394952506951</v>
       </c>
       <c r="H5">
-        <v>4.789012433862396</v>
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>0.76548862857474</v>
+        <v>0.574127438723655</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>10.64943109565036</v>
+        <v>17.56917343216907</v>
       </c>
       <c r="C6">
-        <v>249.0321523839551</v>
+        <v>789.3964070223751</v>
       </c>
       <c r="D6">
-        <v>14.20191255247596</v>
+        <v>24.13531616499252</v>
       </c>
       <c r="E6">
-        <v>0.7741271154704554</v>
+        <v>0.3236340906910181</v>
       </c>
       <c r="F6">
-        <v>0.7553043750929934</v>
+        <v>0.2672702649152696</v>
       </c>
       <c r="G6">
-        <v>22.24528501761244</v>
+        <v>38.33727603024025</v>
       </c>
       <c r="H6">
-        <v>8.586047109788218</v>
+        <v>13.83912052939468</v>
       </c>
       <c r="I6">
-        <v>0.7748371798272269</v>
+        <v>0.3236340906910181</v>
       </c>
     </row>
   </sheetData>
@@ -1382,176 +1544,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>9.744504761904759</v>
+        <v>10.18400410812769</v>
       </c>
       <c r="C2">
-        <v>174.6017692153439</v>
+        <v>189.9897117553252</v>
       </c>
       <c r="D2">
-        <v>13.21369627376624</v>
+        <v>13.78367555317976</v>
       </c>
       <c r="E2">
-        <v>0.8962613956400378</v>
+        <v>0.8871187409565098</v>
       </c>
       <c r="F2">
-        <v>0.8876165119433743</v>
+        <v>0.8532543632434627</v>
       </c>
       <c r="G2">
-        <v>56.14016639137427</v>
+        <v>61.13097625092665</v>
       </c>
       <c r="H2">
-        <v>8.945161111110981</v>
+        <v>7.830349026907371</v>
       </c>
       <c r="I2">
-        <v>0.8962613956400378</v>
+        <v>0.8871187409565098</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>2.996882539682586</v>
+        <v>7.668926701638179</v>
       </c>
       <c r="C3">
-        <v>12.10389356684306</v>
+        <v>137.1628170144274</v>
       </c>
       <c r="D3">
-        <v>3.479065042054123</v>
+        <v>11.71165304363254</v>
       </c>
       <c r="E3">
-        <v>0.9240220654859893</v>
+        <v>0.139008661028941</v>
       </c>
       <c r="F3">
-        <v>0.9176905709431551</v>
+        <v>-0.1192887406623766</v>
       </c>
       <c r="G3">
-        <v>4.85607386447903</v>
+        <v>15.07332819570342</v>
       </c>
       <c r="H3">
-        <v>3.131877777777873</v>
+        <v>4.656081911799802</v>
       </c>
       <c r="I3">
-        <v>0.9240220654859893</v>
+        <v>0.1390086610289412</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>10.21884021164004</v>
+        <v>33.34258327838067</v>
       </c>
       <c r="C4">
-        <v>141.4562546553184</v>
+        <v>2086.174194799422</v>
       </c>
       <c r="D4">
-        <v>11.89353835724754</v>
+        <v>45.67465593520571</v>
       </c>
       <c r="E4">
-        <v>0.9393952327056326</v>
+        <v>0.1062105954988986</v>
       </c>
       <c r="F4">
-        <v>0.934344835431102</v>
+        <v>-0.1619262258514318</v>
       </c>
       <c r="G4">
-        <v>4.368872825302105</v>
+        <v>16.7996861714309</v>
       </c>
       <c r="H4">
-        <v>10.70506666666506</v>
+        <v>22.61631116938514</v>
       </c>
       <c r="I4">
-        <v>0.9393952327056326</v>
+        <v>0.1062105954988986</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>6.1551809523809</v>
+        <v>6.724952823598907</v>
       </c>
       <c r="C5">
-        <v>96.16453862328039</v>
+        <v>103.3948511812794</v>
       </c>
       <c r="D5">
-        <v>9.806351952855882</v>
+        <v>10.16832587898713</v>
       </c>
       <c r="E5">
-        <v>0.7884517419203456</v>
+        <v>0.7725460863750298</v>
       </c>
       <c r="F5">
-        <v>0.7708227204137078</v>
+        <v>0.7043099122875387</v>
       </c>
       <c r="G5">
-        <v>9.099110063463067</v>
+        <v>9.331852024183938</v>
       </c>
       <c r="H5">
-        <v>4.25</v>
+        <v>3.850313105553319</v>
       </c>
       <c r="I5">
-        <v>0.7884517419203456</v>
+        <v>0.7725460863750298</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>7.27885211640207</v>
+        <v>14.48011672793636</v>
       </c>
       <c r="C6">
-        <v>106.0816140151965</v>
+        <v>629.1803936876136</v>
       </c>
       <c r="D6">
-        <v>9.598162906480946</v>
+        <v>20.33457760275129</v>
       </c>
       <c r="E6">
-        <v>0.8870326089380014</v>
+        <v>0.4762210209648448</v>
       </c>
       <c r="F6">
-        <v>0.8776186596828348</v>
+        <v>0.3190873272542982</v>
       </c>
       <c r="G6">
-        <v>18.61605578615462</v>
+        <v>25.58396066056122</v>
       </c>
       <c r="H6">
-        <v>6.758026388888479</v>
+        <v>9.738263803411408</v>
       </c>
       <c r="I6">
-        <v>0.8870326089380014</v>
+        <v>0.4762210209648448</v>
       </c>
     </row>
   </sheetData>
@@ -1566,176 +1728,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>5.547003887826607</v>
+        <v>27.70739324299376</v>
       </c>
       <c r="C2">
-        <v>141.3121283968491</v>
+        <v>1454.16764252894</v>
       </c>
       <c r="D2">
-        <v>11.88747779795399</v>
+        <v>38.1335500908182</v>
       </c>
       <c r="E2">
-        <v>0.9160402380519714</v>
+        <v>0.1360149303222999</v>
       </c>
       <c r="F2">
-        <v>0.9090435912229691</v>
+        <v>-0.1231805905810099</v>
       </c>
       <c r="G2">
-        <v>32.57685910751209</v>
+        <v>133.9881443826817</v>
       </c>
       <c r="H2">
-        <v>0.01996302596227473</v>
+        <v>21.87642648980349</v>
       </c>
       <c r="I2">
-        <v>0.9188843216893332</v>
+        <v>0.1360149303223001</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>1.103320129706783</v>
+        <v>9.230217882112072</v>
       </c>
       <c r="C3">
-        <v>4.993944690047625</v>
+        <v>157.7967482820635</v>
       </c>
       <c r="D3">
-        <v>2.234713558836484</v>
+        <v>12.56171756894986</v>
       </c>
       <c r="E3">
-        <v>0.9686522687487583</v>
+        <v>0.009486415153149741</v>
       </c>
       <c r="F3">
-        <v>0.9660399578111548</v>
+        <v>-0.2876676603009054</v>
       </c>
       <c r="G3">
-        <v>1.556304175908757</v>
+        <v>17.56462955776416</v>
       </c>
       <c r="H3">
-        <v>0.004925863845340217</v>
+        <v>6.969089569453757</v>
       </c>
       <c r="I3">
-        <v>0.9687861808663898</v>
+        <v>0.00948641515314963</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>2.964023435646182</v>
+        <v>32.09597830566354</v>
       </c>
       <c r="C4">
-        <v>42.20397466564071</v>
+        <v>2333.922165194635</v>
       </c>
       <c r="D4">
-        <v>6.496458624946419</v>
+        <v>48.31068375830169</v>
       </c>
       <c r="E4">
-        <v>0.9819183529937157</v>
+        <v>6.676940906247264E-05</v>
       </c>
       <c r="F4">
-        <v>0.9804115490765253</v>
+        <v>-0.2999131997682187</v>
       </c>
       <c r="G4">
-        <v>1.066088054274457</v>
+        <v>16.63859364620697</v>
       </c>
       <c r="H4">
-        <v>0.007191736280468319</v>
+        <v>22.53272535000156</v>
       </c>
       <c r="I4">
-        <v>0.9821539730635134</v>
+        <v>6.676940906247264E-05</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>3.795172832343855</v>
+        <v>15.29171221504644</v>
       </c>
       <c r="C5">
-        <v>87.28676004046827</v>
+        <v>405.4865126565633</v>
       </c>
       <c r="D5">
-        <v>9.342738358771921</v>
+        <v>20.13669567373364</v>
       </c>
       <c r="E5">
-        <v>0.8079815875546916</v>
+        <v>0.1079875528407799</v>
       </c>
       <c r="F5">
-        <v>0.7919800531842492</v>
+        <v>-0.1596161813069863</v>
       </c>
       <c r="G5">
-        <v>6.130674094144062</v>
+        <v>30.75121062888524</v>
       </c>
       <c r="H5">
-        <v>0.007198414576095047</v>
+        <v>12.7769672298138</v>
       </c>
       <c r="I5">
-        <v>0.8105557421850719</v>
+        <v>0.10798755284078</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>3.352380071380857</v>
+        <v>21.08132541145396</v>
       </c>
       <c r="C6">
-        <v>68.94920194825141</v>
+        <v>1087.843267165551</v>
       </c>
       <c r="D6">
-        <v>7.490347085127204</v>
+        <v>29.78566177295085</v>
       </c>
       <c r="E6">
-        <v>0.9186481118372842</v>
+        <v>0.06338891693132301</v>
       </c>
       <c r="F6">
-        <v>0.9118687878237246</v>
+        <v>-0.2175944079892801</v>
       </c>
       <c r="G6">
-        <v>10.33248135795984</v>
+        <v>49.73564455388451</v>
       </c>
       <c r="H6">
-        <v>0.009819760166044578</v>
+        <v>16.03880215976815</v>
       </c>
       <c r="I6">
-        <v>0.9200950544510771</v>
+        <v>0.06338891693132304</v>
       </c>
     </row>
   </sheetData>
@@ -1750,176 +1912,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>6.385833333333335</v>
+        <v>24.10753027245121</v>
       </c>
       <c r="C2">
-        <v>139.9965470238095</v>
+        <v>1136.101462228707</v>
       </c>
       <c r="D2">
-        <v>11.83201365042356</v>
+        <v>33.70610422799863</v>
       </c>
       <c r="E2">
-        <v>0.9168218829125843</v>
+        <v>0.3249920626087158</v>
       </c>
       <c r="F2">
-        <v>0.9098903731552996</v>
+        <v>0.2687414011594421</v>
       </c>
       <c r="G2">
-        <v>30.71379985486174</v>
+        <v>91.66700786904762</v>
       </c>
       <c r="H2">
-        <v>0.8333333333333357</v>
+        <v>15.17144749610551</v>
       </c>
       <c r="I2">
-        <v>0.9173606543729681</v>
+        <v>0.3894790409600025</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>1.738095238095237</v>
+        <v>8.859216086972451</v>
       </c>
       <c r="C3">
-        <v>7.060634920634918</v>
+        <v>158.0302394259915</v>
       </c>
       <c r="D3">
-        <v>2.657185526197769</v>
+        <v>12.57100789220942</v>
       </c>
       <c r="E3">
-        <v>0.9556793477516298</v>
+        <v>0.008020756623934089</v>
       </c>
       <c r="F3">
-        <v>0.9519859600642656</v>
+        <v>-0.07464418032407139</v>
       </c>
       <c r="G3">
-        <v>2.401144235243257</v>
+        <v>16.91965977373152</v>
       </c>
       <c r="H3">
-        <v>0.7499999999999929</v>
+        <v>7.26766547681919</v>
       </c>
       <c r="I3">
-        <v>0.9558958453142707</v>
+        <v>0.01422470829512235</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>6.759285714285718</v>
+        <v>182.298092612082</v>
       </c>
       <c r="C4">
-        <v>87.81028650793662</v>
+        <v>35566.65742346342</v>
       </c>
       <c r="D4">
-        <v>9.370714300838364</v>
+        <v>188.5912442916251</v>
       </c>
       <c r="E4">
-        <v>0.9623790266974587</v>
+        <v>-14.23799001917405</v>
       </c>
       <c r="F4">
-        <v>0.9592439455889136</v>
+        <v>-15.50782252077188</v>
       </c>
       <c r="G4">
-        <v>2.454784806808297</v>
+        <v>67.54990255135532</v>
       </c>
       <c r="H4">
-        <v>5.683333333333337</v>
+        <v>192.8329852518807</v>
       </c>
       <c r="I4">
-        <v>0.9625806183610094</v>
+        <v>6.49367494331976E-06</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>5.094999999999998</v>
+        <v>12.23250900181676</v>
       </c>
       <c r="C5">
-        <v>91.03139563492061</v>
+        <v>248.880094989379</v>
       </c>
       <c r="D5">
-        <v>9.541037450661255</v>
+        <v>15.77593404491091</v>
       </c>
       <c r="E5">
-        <v>0.7997439237704067</v>
+        <v>0.4524993171135955</v>
       </c>
       <c r="F5">
-        <v>0.7830559174179406</v>
+        <v>0.4068742602063952</v>
       </c>
       <c r="G5">
-        <v>7.357244732313917</v>
+        <v>16.02764055785559</v>
       </c>
       <c r="H5">
-        <v>0.62083333333333</v>
+        <v>7.75906641742332</v>
       </c>
       <c r="I5">
-        <v>0.799940969249874</v>
+        <v>0.5691504293723822</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>4.994553571428572</v>
+        <v>56.87433699333061</v>
       </c>
       <c r="C6">
-        <v>81.47471602182542</v>
+        <v>9277.417305026873</v>
       </c>
       <c r="D6">
-        <v>8.350237732030237</v>
+        <v>62.66107261418601</v>
       </c>
       <c r="E6">
-        <v>0.9086560452830199</v>
+        <v>-3.36311947070695</v>
       </c>
       <c r="F6">
-        <v>0.901044049056605</v>
+        <v>-3.726712759932529</v>
       </c>
       <c r="G6">
-        <v>10.7317434073068</v>
+        <v>48.04105268799751</v>
       </c>
       <c r="H6">
-        <v>1.971874999999999</v>
+        <v>55.75779116055718</v>
       </c>
       <c r="I6">
-        <v>0.9089445218245306</v>
+        <v>0.2432151680756126</v>
       </c>
     </row>
   </sheetData>
@@ -1934,176 +2096,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>29.58285714285715</v>
+        <v>19.90424533527296</v>
       </c>
       <c r="C2">
-        <v>1683.093485714286</v>
+        <v>739.1535231056032</v>
       </c>
       <c r="D2">
-        <v>41.02552236979178</v>
+        <v>27.18737801086385</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.5608363234844826</v>
       </c>
       <c r="F2">
-        <v>-0.08333333333333326</v>
+        <v>0.5242393504415228</v>
       </c>
       <c r="G2">
-        <v>140.2043443286067</v>
+        <v>73.12252338226155</v>
       </c>
       <c r="H2">
-        <v>21.79</v>
+        <v>12.38887325851016</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>0.627954300240959</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>9.354081632653058</v>
+        <v>14.93563361960503</v>
       </c>
       <c r="C3">
-        <v>159.3080102040817</v>
+        <v>280.9378681491963</v>
       </c>
       <c r="D3">
-        <v>12.62172770281793</v>
+        <v>16.76120127404943</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>-0.7634886518844886</v>
       </c>
       <c r="F3">
-        <v>-0.08333333333333326</v>
+        <v>-0.9104460395415293</v>
       </c>
       <c r="G3">
-        <v>17.74311782890865</v>
+        <v>25.28355525915003</v>
       </c>
       <c r="H3">
-        <v>7.064285714285703</v>
+        <v>12.74075791853362</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-0.2376284328775833</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>32.10306122448979</v>
+        <v>60.16787149107972</v>
       </c>
       <c r="C4">
-        <v>2334.078010204082</v>
+        <v>4843.972436877133</v>
       </c>
       <c r="D4">
-        <v>48.31229667697534</v>
+        <v>69.59865255072927</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>-1.075325852735143</v>
       </c>
       <c r="F4">
-        <v>-0.08333333333333326</v>
+        <v>-1.248269673796405</v>
       </c>
       <c r="G4">
-        <v>16.6410616884347</v>
+        <v>25.61801496017499</v>
       </c>
       <c r="H4">
-        <v>22.53571428571428</v>
+        <v>50.75652110070396</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>-0.4684887862410099</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>16.16020408163265</v>
+        <v>11.81222930856601</v>
       </c>
       <c r="C5">
-        <v>454.5749489795918</v>
+        <v>193.0155130603527</v>
       </c>
       <c r="D5">
-        <v>21.32076333013412</v>
+        <v>13.89300230549008</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>0.5753934230348049</v>
       </c>
       <c r="F5">
-        <v>-0.08333333333333326</v>
+        <v>0.5400095416210386</v>
       </c>
       <c r="G5">
-        <v>32.8731008901733</v>
+        <v>18.39019652709208</v>
       </c>
       <c r="H5">
-        <v>13.29285714285713</v>
+        <v>13.0256948339919</v>
       </c>
       <c r="I5">
-        <v>-2.220446049250313E-16</v>
+        <v>0.7306836652249162</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>21.80005102040816</v>
+        <v>26.70499493863093</v>
       </c>
       <c r="C6">
-        <v>1157.76361377551</v>
+        <v>1514.269835298071</v>
       </c>
       <c r="D6">
-        <v>30.8200775199298</v>
+        <v>31.86005853528316</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>-0.1756461895250861</v>
       </c>
       <c r="F6">
-        <v>-0.08333333333333326</v>
+        <v>-0.2736167053188433</v>
       </c>
       <c r="G6">
-        <v>51.86540618403083</v>
+        <v>35.60357253216966</v>
       </c>
       <c r="H6">
-        <v>16.17071428571428</v>
+        <v>22.22796177793491</v>
       </c>
       <c r="I6">
-        <v>-5.551115123125783E-17</v>
+        <v>0.1631301865868205</v>
       </c>
     </row>
   </sheetData>
@@ -2118,176 +2280,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>11.30476428571428</v>
+        <v>11.18523809523809</v>
       </c>
       <c r="C2">
-        <v>225.6083918291567</v>
+        <v>201.3859261904761</v>
       </c>
       <c r="D2">
-        <v>15.02026603722972</v>
+        <v>14.19105091917002</v>
       </c>
       <c r="E2">
-        <v>0.865956113701307</v>
+        <v>0.8803477478228072</v>
       </c>
       <c r="F2">
-        <v>0.8547857898430826</v>
+        <v>0.8703767268080411</v>
       </c>
       <c r="G2">
-        <v>55.43836192495155</v>
+        <v>58.07192754245103</v>
       </c>
       <c r="H2">
-        <v>8.551895833333329</v>
+        <v>9.435833333333328</v>
       </c>
       <c r="I2">
-        <v>0.870053822148988</v>
+        <v>0.8803477478228072</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>4.348476190476187</v>
+        <v>4.207142857142858</v>
       </c>
       <c r="C3">
-        <v>30.45792862003967</v>
+        <v>23.39107142857144</v>
       </c>
       <c r="D3">
-        <v>5.518870230404016</v>
+        <v>4.83643168343888</v>
       </c>
       <c r="E3">
-        <v>0.8088110661791487</v>
+        <v>0.8531707765440903</v>
       </c>
       <c r="F3">
-        <v>0.7928786550274111</v>
+        <v>0.8409350079227645</v>
       </c>
       <c r="G3">
-        <v>7.648256241692383</v>
+        <v>7.268140300799806</v>
       </c>
       <c r="H3">
-        <v>3.654999999999987</v>
+        <v>3.524999999999999</v>
       </c>
       <c r="I3">
-        <v>0.8097421870952792</v>
+        <v>0.8531707765440903</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>17.01513988095239</v>
+        <v>15.00714285714286</v>
       </c>
       <c r="C4">
-        <v>425.9112810809776</v>
+        <v>336.815773809524</v>
       </c>
       <c r="D4">
-        <v>20.63761810580324</v>
+        <v>18.35254134471638</v>
       </c>
       <c r="E4">
-        <v>0.8175248302674606</v>
+        <v>0.8556964367356024</v>
       </c>
       <c r="F4">
-        <v>0.8023185661230823</v>
+        <v>0.8436711397969026</v>
       </c>
       <c r="G4">
-        <v>7.808682415642464</v>
+        <v>6.80814351818554</v>
       </c>
       <c r="H4">
-        <v>15.90499999999994</v>
+        <v>15.44583333333333</v>
       </c>
       <c r="I4">
-        <v>0.8177246363479393</v>
+        <v>0.8556964367356024</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>7.113553571428571</v>
+        <v>7.223809523809522</v>
       </c>
       <c r="C5">
-        <v>108.1679850183531</v>
+        <v>105.027619047619</v>
       </c>
       <c r="D5">
-        <v>10.40038388802803</v>
+        <v>10.24829834887817</v>
       </c>
       <c r="E5">
-        <v>0.7620458732687239</v>
+        <v>0.7689542301365704</v>
       </c>
       <c r="F5">
-        <v>0.7422163627077842</v>
+        <v>0.7497004159812846</v>
       </c>
       <c r="G5">
-        <v>12.66473414599422</v>
+        <v>11.21539909324933</v>
       </c>
       <c r="H5">
-        <v>5.110416666666669</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>0.7673903392117379</v>
+        <v>0.7689542301365704</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>9.945483482142858</v>
+        <v>9.405833333333334</v>
       </c>
       <c r="C6">
-        <v>197.5363966371318</v>
+        <v>166.6550976190477</v>
       </c>
       <c r="D6">
-        <v>12.89428456536625</v>
+        <v>11.90708057405086</v>
       </c>
       <c r="E6">
-        <v>0.81358447085416</v>
+        <v>0.8395422978097675</v>
       </c>
       <c r="F6">
-        <v>0.79804984342534</v>
+        <v>0.8261708226272482</v>
       </c>
       <c r="G6">
-        <v>20.89000868207015</v>
+        <v>20.84090261367143</v>
       </c>
       <c r="H6">
-        <v>8.305578124999982</v>
+        <v>8.351666666666663</v>
       </c>
       <c r="I6">
-        <v>0.8162277462009861</v>
+        <v>0.8395422978097675</v>
       </c>
     </row>
   </sheetData>
@@ -2302,176 +2464,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>23.82523809523809</v>
+        <v>11.20179695011338</v>
       </c>
       <c r="C2">
-        <v>1358.989868430335</v>
+        <v>224.7096343972572</v>
       </c>
       <c r="D2">
-        <v>36.8644797661697</v>
+        <v>14.99031802188523</v>
       </c>
       <c r="E2">
-        <v>0.192564239618814</v>
+        <v>0.8664901050924733</v>
       </c>
       <c r="F2">
-        <v>0.1252779262537151</v>
+        <v>0.855364280516846</v>
       </c>
       <c r="G2">
-        <v>89.51563936683232</v>
+        <v>58.90464254253096</v>
       </c>
       <c r="H2">
-        <v>13.88888888888889</v>
+        <v>8.386608544973544</v>
       </c>
       <c r="I2">
-        <v>0.250581756450024</v>
+        <v>0.8678324828815218</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>9.28809523809524</v>
+        <v>4.73816678004534</v>
       </c>
       <c r="C3">
-        <v>153.5173985890652</v>
+        <v>42.66476898952453</v>
       </c>
       <c r="D3">
-        <v>12.39021382337953</v>
+        <v>6.531827385159878</v>
       </c>
       <c r="E3">
-        <v>0.03634852765782681</v>
+        <v>0.7321869193214529</v>
       </c>
       <c r="F3">
-        <v>-0.04395576170402093</v>
+        <v>0.7098691625982405</v>
       </c>
       <c r="G3">
-        <v>17.46387395743525</v>
+        <v>8.831622888899272</v>
       </c>
       <c r="H3">
-        <v>7.044444444444444</v>
+        <v>3.799534920634933</v>
       </c>
       <c r="I3">
-        <v>0.0368868892004296</v>
+        <v>0.7323021588655974</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>35.8015873015873</v>
+        <v>19.56376118154327</v>
       </c>
       <c r="C4">
-        <v>2324.184144620812</v>
+        <v>621.5268394215173</v>
       </c>
       <c r="D4">
-        <v>48.20979303648598</v>
+        <v>24.93044001660455</v>
       </c>
       <c r="E4">
-        <v>0.004238875281809995</v>
+        <v>0.7337163382267701</v>
       </c>
       <c r="F4">
-        <v>-0.07874121844470583</v>
+        <v>0.711526033079001</v>
       </c>
       <c r="G4">
-        <v>17.42832607359704</v>
+        <v>9.410596220698149</v>
       </c>
       <c r="H4">
-        <v>31.50555555555555</v>
+        <v>17.369032539682</v>
       </c>
       <c r="I4">
-        <v>0.02928593934982482</v>
+        <v>0.7337254489870485</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>13.31746031746031</v>
+        <v>7.093999470899462</v>
       </c>
       <c r="C5">
-        <v>386.5201940035274</v>
+        <v>107.2273667275214</v>
       </c>
       <c r="D5">
-        <v>19.66011683595821</v>
+        <v>10.35506478625418</v>
       </c>
       <c r="E5">
-        <v>0.1497107465530833</v>
+        <v>0.7641150992411256</v>
       </c>
       <c r="F5">
-        <v>0.07885330876584018</v>
+        <v>0.7444580241778862</v>
       </c>
       <c r="G5">
-        <v>29.86622669604085</v>
+        <v>11.83427841832139</v>
       </c>
       <c r="H5">
-        <v>8.049999999999997</v>
+        <v>4.789012433862396</v>
       </c>
       <c r="I5">
-        <v>0.215911185649081</v>
+        <v>0.76548862857474</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>20.55809523809524</v>
+        <v>10.64943109565036</v>
       </c>
       <c r="C6">
-        <v>1055.802901410935</v>
+        <v>249.0321523839551</v>
       </c>
       <c r="D6">
-        <v>29.28115086549835</v>
+        <v>14.20191255247596</v>
       </c>
       <c r="E6">
-        <v>0.09571559727788351</v>
+        <v>0.7741271154704554</v>
       </c>
       <c r="F6">
-        <v>0.02035856371770714</v>
+        <v>0.7553043750929934</v>
       </c>
       <c r="G6">
-        <v>38.56851652347636</v>
+        <v>22.24528501761244</v>
       </c>
       <c r="H6">
-        <v>15.12222222222222</v>
+        <v>8.586047109788218</v>
       </c>
       <c r="I6">
-        <v>0.1331664426623398</v>
+        <v>0.7748371798272269</v>
       </c>
     </row>
   </sheetData>
@@ -2486,176 +2648,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>23.82523809523809</v>
+        <v>9.744504761904759</v>
       </c>
       <c r="C2">
-        <v>1358.989868430335</v>
+        <v>174.6017692153439</v>
       </c>
       <c r="D2">
-        <v>36.8644797661697</v>
+        <v>13.21369627376624</v>
       </c>
       <c r="E2">
-        <v>0.192564239618814</v>
+        <v>0.8962613956400378</v>
       </c>
       <c r="F2">
-        <v>0.1252779262537151</v>
+        <v>0.8876165119433743</v>
       </c>
       <c r="G2">
-        <v>89.51563936683232</v>
+        <v>56.14016639137427</v>
       </c>
       <c r="H2">
-        <v>13.88888888888889</v>
+        <v>8.945161111110981</v>
       </c>
       <c r="I2">
-        <v>0.250581756450024</v>
+        <v>0.8962613956400378</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>9.28809523809524</v>
+        <v>2.996882539682586</v>
       </c>
       <c r="C3">
-        <v>153.5173985890652</v>
+        <v>12.10389356684306</v>
       </c>
       <c r="D3">
-        <v>12.39021382337953</v>
+        <v>3.479065042054123</v>
       </c>
       <c r="E3">
-        <v>0.03634852765782681</v>
+        <v>0.9240220654859893</v>
       </c>
       <c r="F3">
-        <v>-0.04395576170402093</v>
+        <v>0.9176905709431551</v>
       </c>
       <c r="G3">
-        <v>17.46387395743525</v>
+        <v>4.85607386447903</v>
       </c>
       <c r="H3">
-        <v>7.044444444444444</v>
+        <v>3.131877777777873</v>
       </c>
       <c r="I3">
-        <v>0.0368868892004296</v>
+        <v>0.9240220654859893</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>35.8015873015873</v>
+        <v>10.21884021164004</v>
       </c>
       <c r="C4">
-        <v>2324.184144620812</v>
+        <v>141.4562546553184</v>
       </c>
       <c r="D4">
-        <v>48.20979303648598</v>
+        <v>11.89353835724754</v>
       </c>
       <c r="E4">
-        <v>0.004238875281809995</v>
+        <v>0.9393952327056326</v>
       </c>
       <c r="F4">
-        <v>-0.07874121844470583</v>
+        <v>0.934344835431102</v>
       </c>
       <c r="G4">
-        <v>17.42832607359704</v>
+        <v>4.368872825302105</v>
       </c>
       <c r="H4">
-        <v>31.50555555555555</v>
+        <v>10.70506666666506</v>
       </c>
       <c r="I4">
-        <v>0.02928593934982482</v>
+        <v>0.9393952327056326</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>13.31746031746031</v>
+        <v>6.1551809523809</v>
       </c>
       <c r="C5">
-        <v>386.5201940035274</v>
+        <v>96.16453862328039</v>
       </c>
       <c r="D5">
-        <v>19.66011683595821</v>
+        <v>9.806351952855882</v>
       </c>
       <c r="E5">
-        <v>0.1497107465530833</v>
+        <v>0.7884517419203456</v>
       </c>
       <c r="F5">
-        <v>0.07885330876584018</v>
+        <v>0.7708227204137078</v>
       </c>
       <c r="G5">
-        <v>29.86622669604085</v>
+        <v>9.099110063463067</v>
       </c>
       <c r="H5">
-        <v>8.049999999999997</v>
+        <v>4.25</v>
       </c>
       <c r="I5">
-        <v>0.215911185649081</v>
+        <v>0.7884517419203456</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>20.55809523809524</v>
+        <v>7.27885211640207</v>
       </c>
       <c r="C6">
-        <v>1055.802901410935</v>
+        <v>106.0816140151965</v>
       </c>
       <c r="D6">
-        <v>29.28115086549835</v>
+        <v>9.598162906480946</v>
       </c>
       <c r="E6">
-        <v>0.09571559727788351</v>
+        <v>0.8870326089380014</v>
       </c>
       <c r="F6">
-        <v>0.02035856371770714</v>
+        <v>0.8776186596828348</v>
       </c>
       <c r="G6">
-        <v>38.56851652347636</v>
+        <v>18.61605578615462</v>
       </c>
       <c r="H6">
-        <v>15.12222222222222</v>
+        <v>6.758026388888479</v>
       </c>
       <c r="I6">
-        <v>0.1331664426623398</v>
+        <v>0.8870326089380014</v>
       </c>
     </row>
   </sheetData>
@@ -2670,176 +2832,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>9.446195671540888</v>
+        <v>5.547003887826607</v>
       </c>
       <c r="C2">
-        <v>192.4685111243765</v>
+        <v>141.3121283968491</v>
       </c>
       <c r="D2">
-        <v>13.87330209879308</v>
+        <v>11.88747779795399</v>
       </c>
       <c r="E2">
-        <v>0.8856459770309817</v>
+        <v>0.9160402380519714</v>
       </c>
       <c r="F2">
-        <v>0.8761164751168968</v>
+        <v>0.9090435912229691</v>
       </c>
       <c r="G2">
-        <v>63.97577783465798</v>
+        <v>32.57685910751209</v>
       </c>
       <c r="H2">
-        <v>5.117490080971982</v>
+        <v>0.01996302596227473</v>
       </c>
       <c r="I2">
-        <v>0.8875182305539248</v>
+        <v>0.9188843216893332</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>6.703953457269698</v>
+        <v>1.103320129706783</v>
       </c>
       <c r="C3">
-        <v>142.6746175357007</v>
+        <v>4.993944690047625</v>
       </c>
       <c r="D3">
-        <v>11.94464807081819</v>
+        <v>2.234713558836484</v>
       </c>
       <c r="E3">
-        <v>0.1044102719447233</v>
+        <v>0.9686522687487583</v>
       </c>
       <c r="F3">
-        <v>0.02977779460678354</v>
+        <v>0.9660399578111548</v>
       </c>
       <c r="G3">
-        <v>14.26744988320347</v>
+        <v>1.556304175908757</v>
       </c>
       <c r="H3">
-        <v>2.823378514546043</v>
+        <v>0.004925863845340217</v>
       </c>
       <c r="I3">
-        <v>0.1237868851464625</v>
+        <v>0.9687861808663898</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>26.73518541278025</v>
+        <v>2.964023435646182</v>
       </c>
       <c r="C4">
-        <v>2598.207069926513</v>
+        <v>42.20397466564071</v>
       </c>
       <c r="D4">
-        <v>50.97261097811759</v>
+        <v>6.496458624946419</v>
       </c>
       <c r="E4">
-        <v>-0.1131620530966473</v>
+        <v>0.9819183529937157</v>
       </c>
       <c r="F4">
-        <v>-0.2059255575213679</v>
+        <v>0.9804115490765253</v>
       </c>
       <c r="G4">
-        <v>15.88588951691986</v>
+        <v>1.066088054274457</v>
       </c>
       <c r="H4">
-        <v>10.09913308669061</v>
+        <v>0.007191736280468319</v>
       </c>
       <c r="I4">
-        <v>0.08419040624466256</v>
+        <v>0.9821539730635134</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>6.362135142658091</v>
+        <v>3.795172832343855</v>
       </c>
       <c r="C5">
-        <v>105.3601690489118</v>
+        <v>87.28676004046827</v>
       </c>
       <c r="D5">
-        <v>10.2645101709196</v>
+        <v>9.342738358771921</v>
       </c>
       <c r="E5">
-        <v>0.7682226676031767</v>
+        <v>0.8079815875546916</v>
       </c>
       <c r="F5">
-        <v>0.7489078899034414</v>
+        <v>0.7919800531842492</v>
       </c>
       <c r="G5">
-        <v>8.703613141130717</v>
+        <v>6.130674094144062</v>
       </c>
       <c r="H5">
-        <v>3.207255368886877</v>
+        <v>0.007198414576095047</v>
       </c>
       <c r="I5">
-        <v>0.7708767769947198</v>
+        <v>0.8105557421850719</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>12.31186742106223</v>
+        <v>3.352380071380857</v>
       </c>
       <c r="C6">
-        <v>759.6775919088756</v>
+        <v>68.94920194825141</v>
       </c>
       <c r="D6">
-        <v>21.76376782966211</v>
+        <v>7.490347085127204</v>
       </c>
       <c r="E6">
-        <v>0.4112792158705586</v>
+        <v>0.9186481118372842</v>
       </c>
       <c r="F6">
-        <v>0.3622191505264385</v>
+        <v>0.9118687878237246</v>
       </c>
       <c r="G6">
-        <v>25.70818259397801</v>
+        <v>10.33248135795984</v>
       </c>
       <c r="H6">
-        <v>5.311814262773879</v>
+        <v>0.009819760166044578</v>
       </c>
       <c r="I6">
-        <v>0.4665930747349424</v>
+        <v>0.9200950544510771</v>
       </c>
     </row>
   </sheetData>
@@ -2854,21 +3016,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -2882,7 +3044,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
@@ -2896,7 +3058,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -2910,7 +3072,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -2934,36 +3096,1140 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>6.385833333333335</v>
+      </c>
+      <c r="C2">
+        <v>139.9965470238095</v>
+      </c>
+      <c r="D2">
+        <v>11.83201365042356</v>
+      </c>
+      <c r="E2">
+        <v>0.9168218829125843</v>
+      </c>
+      <c r="F2">
+        <v>0.9098903731552996</v>
+      </c>
+      <c r="G2">
+        <v>30.71379985486174</v>
+      </c>
+      <c r="H2">
+        <v>0.8333333333333357</v>
+      </c>
+      <c r="I2">
+        <v>0.9173606543729681</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>1.738095238095237</v>
+      </c>
+      <c r="C3">
+        <v>7.060634920634918</v>
+      </c>
+      <c r="D3">
+        <v>2.657185526197769</v>
+      </c>
+      <c r="E3">
+        <v>0.9556793477516298</v>
+      </c>
+      <c r="F3">
+        <v>0.9519859600642656</v>
+      </c>
+      <c r="G3">
+        <v>2.401144235243257</v>
+      </c>
+      <c r="H3">
+        <v>0.7499999999999929</v>
+      </c>
+      <c r="I3">
+        <v>0.9558958453142707</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>6.759285714285718</v>
+      </c>
+      <c r="C4">
+        <v>87.81028650793662</v>
+      </c>
+      <c r="D4">
+        <v>9.370714300838364</v>
+      </c>
+      <c r="E4">
+        <v>0.9623790266974587</v>
+      </c>
+      <c r="F4">
+        <v>0.9592439455889136</v>
+      </c>
+      <c r="G4">
+        <v>2.454784806808297</v>
+      </c>
+      <c r="H4">
+        <v>5.683333333333337</v>
+      </c>
+      <c r="I4">
+        <v>0.9625806183610094</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>5.094999999999998</v>
+      </c>
+      <c r="C5">
+        <v>91.03139563492061</v>
+      </c>
+      <c r="D5">
+        <v>9.541037450661255</v>
+      </c>
+      <c r="E5">
+        <v>0.7997439237704067</v>
+      </c>
+      <c r="F5">
+        <v>0.7830559174179406</v>
+      </c>
+      <c r="G5">
+        <v>7.357244732313917</v>
+      </c>
+      <c r="H5">
+        <v>0.62083333333333</v>
+      </c>
+      <c r="I5">
+        <v>0.799940969249874</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>4.994553571428572</v>
+      </c>
+      <c r="C6">
+        <v>81.47471602182542</v>
+      </c>
+      <c r="D6">
+        <v>8.350237732030237</v>
+      </c>
+      <c r="E6">
+        <v>0.9086560452830199</v>
+      </c>
+      <c r="F6">
+        <v>0.901044049056605</v>
+      </c>
+      <c r="G6">
+        <v>10.7317434073068</v>
+      </c>
+      <c r="H6">
+        <v>1.971874999999999</v>
+      </c>
+      <c r="I6">
+        <v>0.9089445218245306</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>29.58285714285715</v>
+      </c>
+      <c r="C2">
+        <v>1683.093485714286</v>
+      </c>
+      <c r="D2">
+        <v>41.02552236979178</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>-0.08333333333333326</v>
+      </c>
+      <c r="G2">
+        <v>140.2043443286067</v>
+      </c>
+      <c r="H2">
+        <v>21.79</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>9.354081632653058</v>
+      </c>
+      <c r="C3">
+        <v>159.3080102040817</v>
+      </c>
+      <c r="D3">
+        <v>12.62172770281793</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>-0.08333333333333326</v>
+      </c>
+      <c r="G3">
+        <v>17.74311782890865</v>
+      </c>
+      <c r="H3">
+        <v>7.064285714285703</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>32.10306122448979</v>
+      </c>
+      <c r="C4">
+        <v>2334.078010204082</v>
+      </c>
+      <c r="D4">
+        <v>48.31229667697534</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>-0.08333333333333326</v>
+      </c>
+      <c r="G4">
+        <v>16.6410616884347</v>
+      </c>
+      <c r="H4">
+        <v>22.53571428571428</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>16.16020408163265</v>
+      </c>
+      <c r="C5">
+        <v>454.5749489795918</v>
+      </c>
+      <c r="D5">
+        <v>21.32076333013412</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>-0.08333333333333326</v>
+      </c>
+      <c r="G5">
+        <v>32.8731008901733</v>
+      </c>
+      <c r="H5">
+        <v>13.29285714285713</v>
+      </c>
+      <c r="I5">
+        <v>-2.220446049250313E-16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>21.80005102040816</v>
+      </c>
+      <c r="C6">
+        <v>1157.76361377551</v>
+      </c>
+      <c r="D6">
+        <v>30.8200775199298</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>-0.08333333333333326</v>
+      </c>
+      <c r="G6">
+        <v>51.86540618403083</v>
+      </c>
+      <c r="H6">
+        <v>16.17071428571428</v>
+      </c>
+      <c r="I6">
+        <v>-5.551115123125783E-17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>11.30476428571428</v>
+      </c>
+      <c r="C2">
+        <v>225.6083918291567</v>
+      </c>
+      <c r="D2">
+        <v>15.02026603722972</v>
+      </c>
+      <c r="E2">
+        <v>0.865956113701307</v>
+      </c>
+      <c r="F2">
+        <v>0.8547857898430826</v>
+      </c>
+      <c r="G2">
+        <v>55.43836192495155</v>
+      </c>
+      <c r="H2">
+        <v>8.551895833333329</v>
+      </c>
+      <c r="I2">
+        <v>0.870053822148988</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>4.348476190476187</v>
+      </c>
+      <c r="C3">
+        <v>30.45792862003967</v>
+      </c>
+      <c r="D3">
+        <v>5.518870230404016</v>
+      </c>
+      <c r="E3">
+        <v>0.8088110661791487</v>
+      </c>
+      <c r="F3">
+        <v>0.7928786550274111</v>
+      </c>
+      <c r="G3">
+        <v>7.648256241692383</v>
+      </c>
+      <c r="H3">
+        <v>3.654999999999987</v>
+      </c>
+      <c r="I3">
+        <v>0.8097421870952792</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>17.01513988095239</v>
+      </c>
+      <c r="C4">
+        <v>425.9112810809776</v>
+      </c>
+      <c r="D4">
+        <v>20.63761810580324</v>
+      </c>
+      <c r="E4">
+        <v>0.8175248302674606</v>
+      </c>
+      <c r="F4">
+        <v>0.8023185661230823</v>
+      </c>
+      <c r="G4">
+        <v>7.808682415642464</v>
+      </c>
+      <c r="H4">
+        <v>15.90499999999994</v>
+      </c>
+      <c r="I4">
+        <v>0.8177246363479393</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>7.113553571428571</v>
+      </c>
+      <c r="C5">
+        <v>108.1679850183531</v>
+      </c>
+      <c r="D5">
+        <v>10.40038388802803</v>
+      </c>
+      <c r="E5">
+        <v>0.7620458732687239</v>
+      </c>
+      <c r="F5">
+        <v>0.7422163627077842</v>
+      </c>
+      <c r="G5">
+        <v>12.66473414599422</v>
+      </c>
+      <c r="H5">
+        <v>5.110416666666669</v>
+      </c>
+      <c r="I5">
+        <v>0.7673903392117379</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>9.945483482142858</v>
+      </c>
+      <c r="C6">
+        <v>197.5363966371318</v>
+      </c>
+      <c r="D6">
+        <v>12.89428456536625</v>
+      </c>
+      <c r="E6">
+        <v>0.81358447085416</v>
+      </c>
+      <c r="F6">
+        <v>0.79804984342534</v>
+      </c>
+      <c r="G6">
+        <v>20.89000868207015</v>
+      </c>
+      <c r="H6">
+        <v>8.305578124999982</v>
+      </c>
+      <c r="I6">
+        <v>0.8162277462009861</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>23.82523809523809</v>
+      </c>
+      <c r="C2">
+        <v>1358.989868430335</v>
+      </c>
+      <c r="D2">
+        <v>36.8644797661697</v>
+      </c>
+      <c r="E2">
+        <v>0.192564239618814</v>
+      </c>
+      <c r="F2">
+        <v>0.1252779262537151</v>
+      </c>
+      <c r="G2">
+        <v>89.51563936683232</v>
+      </c>
+      <c r="H2">
+        <v>13.88888888888889</v>
+      </c>
+      <c r="I2">
+        <v>0.250581756450024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>9.28809523809524</v>
+      </c>
+      <c r="C3">
+        <v>153.5173985890652</v>
+      </c>
+      <c r="D3">
+        <v>12.39021382337953</v>
+      </c>
+      <c r="E3">
+        <v>0.03634852765782681</v>
+      </c>
+      <c r="F3">
+        <v>-0.04395576170402093</v>
+      </c>
+      <c r="G3">
+        <v>17.46387395743525</v>
+      </c>
+      <c r="H3">
+        <v>7.044444444444444</v>
+      </c>
+      <c r="I3">
+        <v>0.0368868892004296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>35.8015873015873</v>
+      </c>
+      <c r="C4">
+        <v>2324.184144620812</v>
+      </c>
+      <c r="D4">
+        <v>48.20979303648598</v>
+      </c>
+      <c r="E4">
+        <v>0.004238875281809995</v>
+      </c>
+      <c r="F4">
+        <v>-0.07874121844470583</v>
+      </c>
+      <c r="G4">
+        <v>17.42832607359704</v>
+      </c>
+      <c r="H4">
+        <v>31.50555555555555</v>
+      </c>
+      <c r="I4">
+        <v>0.02928593934982482</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>13.31746031746031</v>
+      </c>
+      <c r="C5">
+        <v>386.5201940035274</v>
+      </c>
+      <c r="D5">
+        <v>19.66011683595821</v>
+      </c>
+      <c r="E5">
+        <v>0.1497107465530833</v>
+      </c>
+      <c r="F5">
+        <v>0.07885330876584018</v>
+      </c>
+      <c r="G5">
+        <v>29.86622669604085</v>
+      </c>
+      <c r="H5">
+        <v>8.049999999999997</v>
+      </c>
+      <c r="I5">
+        <v>0.215911185649081</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>20.55809523809524</v>
+      </c>
+      <c r="C6">
+        <v>1055.802901410935</v>
+      </c>
+      <c r="D6">
+        <v>29.28115086549835</v>
+      </c>
+      <c r="E6">
+        <v>0.09571559727788351</v>
+      </c>
+      <c r="F6">
+        <v>0.02035856371770714</v>
+      </c>
+      <c r="G6">
+        <v>38.56851652347636</v>
+      </c>
+      <c r="H6">
+        <v>15.12222222222222</v>
+      </c>
+      <c r="I6">
+        <v>0.1331664426623398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>23.82523809523809</v>
+      </c>
+      <c r="C2">
+        <v>1358.989868430335</v>
+      </c>
+      <c r="D2">
+        <v>36.8644797661697</v>
+      </c>
+      <c r="E2">
+        <v>0.192564239618814</v>
+      </c>
+      <c r="F2">
+        <v>0.1252779262537151</v>
+      </c>
+      <c r="G2">
+        <v>89.51563936683232</v>
+      </c>
+      <c r="H2">
+        <v>13.88888888888889</v>
+      </c>
+      <c r="I2">
+        <v>0.250581756450024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>9.28809523809524</v>
+      </c>
+      <c r="C3">
+        <v>153.5173985890652</v>
+      </c>
+      <c r="D3">
+        <v>12.39021382337953</v>
+      </c>
+      <c r="E3">
+        <v>0.03634852765782681</v>
+      </c>
+      <c r="F3">
+        <v>-0.04395576170402093</v>
+      </c>
+      <c r="G3">
+        <v>17.46387395743525</v>
+      </c>
+      <c r="H3">
+        <v>7.044444444444444</v>
+      </c>
+      <c r="I3">
+        <v>0.0368868892004296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>35.8015873015873</v>
+      </c>
+      <c r="C4">
+        <v>2324.184144620812</v>
+      </c>
+      <c r="D4">
+        <v>48.20979303648598</v>
+      </c>
+      <c r="E4">
+        <v>0.004238875281809995</v>
+      </c>
+      <c r="F4">
+        <v>-0.07874121844470583</v>
+      </c>
+      <c r="G4">
+        <v>17.42832607359704</v>
+      </c>
+      <c r="H4">
+        <v>31.50555555555555</v>
+      </c>
+      <c r="I4">
+        <v>0.02928593934982482</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>13.31746031746031</v>
+      </c>
+      <c r="C5">
+        <v>386.5201940035274</v>
+      </c>
+      <c r="D5">
+        <v>19.66011683595821</v>
+      </c>
+      <c r="E5">
+        <v>0.1497107465530833</v>
+      </c>
+      <c r="F5">
+        <v>0.07885330876584018</v>
+      </c>
+      <c r="G5">
+        <v>29.86622669604085</v>
+      </c>
+      <c r="H5">
+        <v>8.049999999999997</v>
+      </c>
+      <c r="I5">
+        <v>0.215911185649081</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>20.55809523809524</v>
+      </c>
+      <c r="C6">
+        <v>1055.802901410935</v>
+      </c>
+      <c r="D6">
+        <v>29.28115086549835</v>
+      </c>
+      <c r="E6">
+        <v>0.09571559727788351</v>
+      </c>
+      <c r="F6">
+        <v>0.02035856371770714</v>
+      </c>
+      <c r="G6">
+        <v>38.56851652347636</v>
+      </c>
+      <c r="H6">
+        <v>15.12222222222222</v>
+      </c>
+      <c r="I6">
+        <v>0.1331664426623398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2">
+        <v>9.446195671540888</v>
+      </c>
+      <c r="C2">
+        <v>192.4685111243765</v>
+      </c>
+      <c r="D2">
+        <v>13.87330209879308</v>
+      </c>
+      <c r="E2">
+        <v>0.8856459770309817</v>
+      </c>
+      <c r="F2">
+        <v>0.8761164751168968</v>
+      </c>
+      <c r="G2">
+        <v>63.97577783465798</v>
+      </c>
+      <c r="H2">
+        <v>5.117490080971982</v>
+      </c>
+      <c r="I2">
+        <v>0.8875182305539248</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3">
+        <v>6.703953457269698</v>
+      </c>
+      <c r="C3">
+        <v>142.6746175357007</v>
+      </c>
+      <c r="D3">
+        <v>11.94464807081819</v>
+      </c>
+      <c r="E3">
+        <v>0.1044102719447233</v>
+      </c>
+      <c r="F3">
+        <v>0.02977779460678354</v>
+      </c>
+      <c r="G3">
+        <v>14.26744988320347</v>
+      </c>
+      <c r="H3">
+        <v>2.823378514546043</v>
+      </c>
+      <c r="I3">
+        <v>0.1237868851464625</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>26.73518541278025</v>
+      </c>
+      <c r="C4">
+        <v>2598.207069926513</v>
+      </c>
+      <c r="D4">
+        <v>50.97261097811759</v>
+      </c>
+      <c r="E4">
+        <v>-0.1131620530966473</v>
+      </c>
+      <c r="F4">
+        <v>-0.2059255575213679</v>
+      </c>
+      <c r="G4">
+        <v>15.88588951691986</v>
+      </c>
+      <c r="H4">
+        <v>10.09913308669061</v>
+      </c>
+      <c r="I4">
+        <v>0.08419040624466256</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>6.362135142658091</v>
+      </c>
+      <c r="C5">
+        <v>105.3601690489118</v>
+      </c>
+      <c r="D5">
+        <v>10.2645101709196</v>
+      </c>
+      <c r="E5">
+        <v>0.7682226676031767</v>
+      </c>
+      <c r="F5">
+        <v>0.7489078899034414</v>
+      </c>
+      <c r="G5">
+        <v>8.703613141130717</v>
+      </c>
+      <c r="H5">
+        <v>3.207255368886877</v>
+      </c>
+      <c r="I5">
+        <v>0.7708767769947198</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>12.31186742106223</v>
+      </c>
+      <c r="C6">
+        <v>759.6775919088756</v>
+      </c>
+      <c r="D6">
+        <v>21.76376782966211</v>
+      </c>
+      <c r="E6">
+        <v>0.4112792158705586</v>
+      </c>
+      <c r="F6">
+        <v>0.3622191505264385</v>
+      </c>
+      <c r="G6">
+        <v>25.70818259397801</v>
+      </c>
+      <c r="H6">
+        <v>5.311814262773879</v>
+      </c>
+      <c r="I6">
+        <v>0.4665930747349424</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>37</v>
       </c>
       <c r="B2">
         <v>10.08782696009768</v>
@@ -2992,7 +4258,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>1.136230829833945</v>
@@ -3021,7 +4287,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>2.983787378796376</v>
@@ -3050,7 +4316,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>3.877356776757563</v>
@@ -3079,7 +4345,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>4.52130048637139</v>
@@ -3118,36 +4384,36 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>17.95974911175558</v>
@@ -3176,7 +4442,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>8.696079553061745</v>
@@ -3205,7 +4471,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>33.11990447568959</v>
@@ -3234,7 +4500,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>10.56976793335318</v>
@@ -3263,7 +4529,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>17.58637526846502</v>
@@ -3302,36 +4568,36 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>17.95978215412796</v>
@@ -3360,7 +4626,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>8.696083677245394</v>
@@ -3389,7 +4655,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>33.11988792692743</v>
@@ -3418,7 +4684,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>10.56978718705986</v>
@@ -3447,7 +4713,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>17.58638523634016</v>
@@ -3486,36 +4752,36 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>17.95975043968054</v>
@@ -3544,7 +4810,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>8.696082729744493</v>
@@ -3573,7 +4839,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>33.11989984783138</v>
@@ -3602,7 +4868,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>10.56976959922311</v>
@@ -3631,7 +4897,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>17.58637565411988</v>
@@ -3670,36 +4936,36 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>17.95977618491867</v>
@@ -3728,7 +4994,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>8.696084810296183</v>
@@ -3757,7 +5023,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>33.11988844469191</v>
@@ -3786,7 +5052,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>10.56978426526622</v>
@@ -3815,7 +5081,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>17.58638342629325</v>
@@ -3854,176 +5120,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>10.18400410812769</v>
+        <v>17.57558243910309</v>
       </c>
       <c r="C2">
-        <v>189.9897117553252</v>
+        <v>471.6994952662943</v>
       </c>
       <c r="D2">
-        <v>13.78367555317976</v>
+        <v>21.71864395551192</v>
       </c>
       <c r="E2">
-        <v>0.8871187409565098</v>
+        <v>0.7197425459310656</v>
       </c>
       <c r="F2">
-        <v>0.8532543632434627</v>
+        <v>0.6963877580919877</v>
       </c>
       <c r="G2">
-        <v>61.13097625092665</v>
+        <v>102.9482028406972</v>
       </c>
       <c r="H2">
-        <v>7.830349026907371</v>
+        <v>14.69892059121153</v>
       </c>
       <c r="I2">
-        <v>0.8871187409565098</v>
+        <v>0.7200865743816629</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>7.668926701638179</v>
+        <v>7.688261223134083</v>
       </c>
       <c r="C3">
-        <v>137.1628170144274</v>
+        <v>170.5347770923641</v>
       </c>
       <c r="D3">
-        <v>11.71165304363254</v>
+        <v>13.05889647299358</v>
       </c>
       <c r="E3">
-        <v>0.139008661028941</v>
+        <v>-0.07047208030469032</v>
       </c>
       <c r="F3">
-        <v>-0.1192887406623766</v>
+        <v>-0.1596780869967478</v>
       </c>
       <c r="G3">
-        <v>15.07332819570342</v>
+        <v>16.31690754732949</v>
       </c>
       <c r="H3">
-        <v>4.656081911799802</v>
+        <v>3.656045849813388</v>
       </c>
       <c r="I3">
-        <v>0.1390086610289412</v>
+        <v>-0.00208515413196797</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>33.34258327838067</v>
+        <v>29.10473155618492</v>
       </c>
       <c r="C4">
-        <v>2086.174194799422</v>
+        <v>2551.394555507617</v>
       </c>
       <c r="D4">
-        <v>45.67465593520571</v>
+        <v>50.51133096155373</v>
       </c>
       <c r="E4">
-        <v>0.1062105954988986</v>
+        <v>-0.09310594776758685</v>
       </c>
       <c r="F4">
-        <v>-0.1619262258514318</v>
+        <v>-0.1841981100815524</v>
       </c>
       <c r="G4">
-        <v>16.7996861714309</v>
+        <v>16.40328155860542</v>
       </c>
       <c r="H4">
-        <v>22.61631116938514</v>
+        <v>16.05000000000001</v>
       </c>
       <c r="I4">
-        <v>0.1062105954988986</v>
+        <v>-0.02114552817064341</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>6.724952823598907</v>
+        <v>10.71747962997509</v>
       </c>
       <c r="C5">
-        <v>103.3948511812794</v>
+        <v>195.444764653271</v>
       </c>
       <c r="D5">
-        <v>10.16832587898713</v>
+        <v>13.9801561026074</v>
       </c>
       <c r="E5">
-        <v>0.7725460863750298</v>
+        <v>0.5700494162909855</v>
       </c>
       <c r="F5">
-        <v>0.7043099122875387</v>
+        <v>0.534220200981901</v>
       </c>
       <c r="G5">
-        <v>9.331852024183938</v>
+        <v>15.75384120717569</v>
       </c>
       <c r="H5">
-        <v>3.850313105553319</v>
+        <v>9.837635580519869</v>
       </c>
       <c r="I5">
-        <v>0.7725460863750298</v>
+        <v>0.5734645982343662</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>14.48011672793636</v>
+        <v>16.2715137120993</v>
       </c>
       <c r="C6">
-        <v>629.1803936876136</v>
+        <v>847.2683981298865</v>
       </c>
       <c r="D6">
-        <v>20.33457760275129</v>
+        <v>24.81725687316666</v>
       </c>
       <c r="E6">
-        <v>0.4762210209648448</v>
+        <v>0.2815534835374435</v>
       </c>
       <c r="F6">
-        <v>0.3190873272542982</v>
+        <v>0.2216829404988971</v>
       </c>
       <c r="G6">
-        <v>25.58396066056122</v>
+        <v>37.85555828845195</v>
       </c>
       <c r="H6">
-        <v>9.738263803411408</v>
+        <v>11.0606505053862</v>
       </c>
       <c r="I6">
-        <v>0.4762210209648448</v>
+        <v>0.3175801225783544</v>
       </c>
     </row>
   </sheetData>
@@ -4038,176 +5304,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>27.70739324299376</v>
+        <v>29.02302618033499</v>
       </c>
       <c r="C2">
-        <v>1454.16764252894</v>
+        <v>2468.627031331897</v>
       </c>
       <c r="D2">
-        <v>38.1335500908182</v>
+        <v>49.6852798254362</v>
       </c>
       <c r="E2">
-        <v>0.1360149303222999</v>
+        <v>-0.4667200914774139</v>
       </c>
       <c r="F2">
-        <v>-0.1231805905810099</v>
+        <v>-0.5889467657671983</v>
       </c>
       <c r="G2">
-        <v>133.9881443826817</v>
+        <v>86.81251050841237</v>
       </c>
       <c r="H2">
-        <v>21.87642648980349</v>
+        <v>12.67138259041958</v>
       </c>
       <c r="I2">
-        <v>0.1360149303223001</v>
+        <v>-0.2805300512685571</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>9.230217882112072</v>
+        <v>7.98719930545519</v>
       </c>
       <c r="C3">
-        <v>157.7967482820635</v>
+        <v>181.1869010248145</v>
       </c>
       <c r="D3">
-        <v>12.56171756894986</v>
+        <v>13.46056837673709</v>
       </c>
       <c r="E3">
-        <v>0.009486415153149741</v>
+        <v>-0.137337041575655</v>
       </c>
       <c r="F3">
-        <v>-0.2876676603009054</v>
+        <v>-0.2321151283736262</v>
       </c>
       <c r="G3">
-        <v>17.56462955776416</v>
+        <v>17.09435623689846</v>
       </c>
       <c r="H3">
-        <v>6.969089569453757</v>
+        <v>3.83654083060609</v>
       </c>
       <c r="I3">
-        <v>0.00948641515314963</v>
+        <v>0.007181389337885924</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>32.09597830566354</v>
+        <v>29.62569832963566</v>
       </c>
       <c r="C4">
-        <v>2333.922165194635</v>
+        <v>2557.005530932233</v>
       </c>
       <c r="D4">
-        <v>48.31068375830169</v>
+        <v>50.56684220842975</v>
       </c>
       <c r="E4">
-        <v>6.676940906247264E-05</v>
+        <v>-0.09550988431130403</v>
       </c>
       <c r="F4">
-        <v>-0.2999131997682187</v>
+        <v>-0.1868023746705794</v>
       </c>
       <c r="G4">
-        <v>16.63859364620697</v>
+        <v>16.62434963563749</v>
       </c>
       <c r="H4">
-        <v>22.53272535000156</v>
+        <v>16.05000000000001</v>
       </c>
       <c r="I4">
-        <v>6.676940906247264E-05</v>
+        <v>-0.0112969191371759</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>15.29171221504644</v>
+        <v>14.54411275022233</v>
       </c>
       <c r="C5">
-        <v>405.4865126565633</v>
+        <v>465.1066169338093</v>
       </c>
       <c r="D5">
-        <v>20.13669567373364</v>
+        <v>21.56633063211749</v>
       </c>
       <c r="E5">
-        <v>0.1079875528407799</v>
+        <v>-0.02316816616898598</v>
       </c>
       <c r="F5">
-        <v>-0.1596161813069863</v>
+        <v>-0.1084321800164014</v>
       </c>
       <c r="G5">
-        <v>30.75121062888524</v>
+        <v>32.92265100715431</v>
       </c>
       <c r="H5">
-        <v>12.7769672298138</v>
+        <v>9.409763831879488</v>
       </c>
       <c r="I5">
-        <v>0.10798755284078</v>
+        <v>0.09255589061204739</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>21.08132541145396</v>
+        <v>20.29500914141204</v>
       </c>
       <c r="C6">
-        <v>1087.843267165551</v>
+        <v>1417.981520055688</v>
       </c>
       <c r="D6">
-        <v>29.78566177295085</v>
+        <v>33.81975526068013</v>
       </c>
       <c r="E6">
-        <v>0.06338891693132301</v>
+        <v>-0.1806837958833397</v>
       </c>
       <c r="F6">
-        <v>-0.2175944079892801</v>
+        <v>-0.2790741122069513</v>
       </c>
       <c r="G6">
-        <v>49.73564455388451</v>
+        <v>38.36346684702566</v>
       </c>
       <c r="H6">
-        <v>16.03880215976815</v>
+        <v>10.49192181322629</v>
       </c>
       <c r="I6">
-        <v>0.06338891693132304</v>
+        <v>-0.04802242261394993</v>
       </c>
     </row>
   </sheetData>
@@ -4222,176 +5488,176 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>24.10753027245121</v>
+        <v>17.54773599470262</v>
       </c>
       <c r="C2">
-        <v>1136.101462228707</v>
+        <v>527.6794416927642</v>
       </c>
       <c r="D2">
-        <v>33.70610422799863</v>
+        <v>22.97127427228982</v>
       </c>
       <c r="E2">
-        <v>0.3249920626087158</v>
+        <v>0.6864823931816104</v>
       </c>
       <c r="F2">
-        <v>0.2687414011594421</v>
+        <v>0.6603559259467446</v>
       </c>
       <c r="G2">
-        <v>91.66700786904762</v>
+        <v>120.9773351579284</v>
       </c>
       <c r="H2">
-        <v>15.17144749610551</v>
+        <v>9.883399766959476</v>
       </c>
       <c r="I2">
-        <v>0.3894790409600025</v>
+        <v>0.7200502657784622</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>8.859216086972451</v>
+        <v>8.402487892596605</v>
       </c>
       <c r="C3">
-        <v>158.0302394259915</v>
+        <v>223.3139069413178</v>
       </c>
       <c r="D3">
-        <v>12.57100789220942</v>
+        <v>14.94369120871138</v>
       </c>
       <c r="E3">
-        <v>0.008020756623934089</v>
+        <v>-0.4017745037129103</v>
       </c>
       <c r="F3">
-        <v>-0.07464418032407139</v>
+        <v>-0.5185890456889863</v>
       </c>
       <c r="G3">
-        <v>16.91965977373152</v>
+        <v>18.28151887591551</v>
       </c>
       <c r="H3">
-        <v>7.26766547681919</v>
+        <v>3.957352310113002</v>
       </c>
       <c r="I3">
-        <v>0.01422470829512235</v>
+        <v>-0.08325713135512935</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>182.298092612082</v>
+        <v>29.3968752076566</v>
       </c>
       <c r="C4">
-        <v>35566.65742346342</v>
+        <v>2875.654851574982</v>
       </c>
       <c r="D4">
-        <v>188.5912442916251</v>
+        <v>53.62513264855372</v>
       </c>
       <c r="E4">
-        <v>-14.23799001917405</v>
+        <v>-0.232030308757138</v>
       </c>
       <c r="F4">
-        <v>-15.50782252077188</v>
+        <v>-0.3346995011535663</v>
       </c>
       <c r="G4">
-        <v>67.54990255135532</v>
+        <v>17.0217034305537</v>
       </c>
       <c r="H4">
-        <v>192.8329852518807</v>
+        <v>11.1447284598116</v>
       </c>
       <c r="I4">
-        <v>6.49367494331976E-06</v>
+        <v>-0.06138524754905683</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>12.23250900181676</v>
+        <v>25.1339378238342</v>
       </c>
       <c r="C5">
-        <v>248.880094989379</v>
+        <v>2347.462801876008</v>
       </c>
       <c r="D5">
-        <v>15.77593404491091</v>
+        <v>48.45062230638538</v>
       </c>
       <c r="E5">
-        <v>0.4524993171135955</v>
+        <v>-4.164083078369102</v>
       </c>
       <c r="F5">
-        <v>0.4068742602063952</v>
+        <v>-4.594423334899861</v>
       </c>
       <c r="G5">
-        <v>16.02764055785559</v>
+        <v>67.96000940803145</v>
       </c>
       <c r="H5">
-        <v>7.75906641742332</v>
+        <v>7.79414109206855</v>
       </c>
       <c r="I5">
-        <v>0.5691504293723822</v>
+        <v>-3.387758718696268</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6">
-        <v>56.87433699333061</v>
+        <v>20.1202592296975</v>
       </c>
       <c r="C6">
-        <v>9277.417305026873</v>
+        <v>1493.527750521268</v>
       </c>
       <c r="D6">
-        <v>62.66107261418601</v>
+        <v>34.99768010898507</v>
       </c>
       <c r="E6">
-        <v>-3.36311947070695</v>
+        <v>-1.027851374414385</v>
       </c>
       <c r="F6">
-        <v>-3.726712759932529</v>
+        <v>-1.196838988948917</v>
       </c>
       <c r="G6">
-        <v>48.04105268799751</v>
+        <v>56.06014171810725</v>
       </c>
       <c r="H6">
-        <v>55.75779116055718</v>
+        <v>8.194905407238158</v>
       </c>
       <c r="I6">
-        <v>0.2432151680756126</v>
+        <v>-0.7030877079554979</v>
       </c>
     </row>
   </sheetData>

</xml_diff>